<commit_message>
Update Excel File (edit header row high)
</commit_message>
<xml_diff>
--- a/Budget-Report.xlsx
+++ b/Budget-Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orathai\Desktop\Claude Cowork\Budget Report\25690423\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9508966A-75B0-482C-8BFC-9AEC681FD998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28E645A-F750-4972-964C-A36067B8CB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="จำแนกตามแผนงาน" sheetId="1" r:id="rId1"/>
@@ -1823,26 +1823,26 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2172,17 +2172,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+    </row>
+    <row r="4" spans="1:18" ht="32.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>1</v>
       </c>
@@ -8375,10 +8375,10 @@
       </c>
     </row>
     <row r="115" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A115" s="24" t="s">
+      <c r="A115" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="B115" s="24"/>
+      <c r="B115" s="22"/>
       <c r="C115" s="10">
         <v>220142200</v>
       </c>
@@ -16269,10 +16269,10 @@
       </c>
     </row>
     <row r="256" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A256" s="24" t="s">
+      <c r="A256" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="B256" s="24"/>
+      <c r="B256" s="22"/>
       <c r="C256" s="10">
         <v>76013828.769999996</v>
       </c>
@@ -16323,10 +16323,10 @@
       </c>
     </row>
     <row r="257" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A257" s="25" t="s">
+      <c r="A257" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="B257" s="25"/>
+      <c r="B257" s="23"/>
       <c r="C257" s="12">
         <v>296156028.76999998</v>
       </c>
@@ -16545,10 +16545,10 @@
       </c>
     </row>
     <row r="261" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A261" s="24" t="s">
+      <c r="A261" s="22" t="s">
         <v>510</v>
       </c>
-      <c r="B261" s="24"/>
+      <c r="B261" s="22"/>
       <c r="C261" s="10">
         <v>16725580.18</v>
       </c>
@@ -16599,10 +16599,10 @@
       </c>
     </row>
     <row r="262" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A262" s="25" t="s">
+      <c r="A262" s="23" t="s">
         <v>511</v>
       </c>
-      <c r="B262" s="25"/>
+      <c r="B262" s="23"/>
       <c r="C262" s="12">
         <v>312881608.94999999</v>
       </c>
@@ -16821,10 +16821,10 @@
       </c>
     </row>
     <row r="266" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A266" s="24" t="s">
+      <c r="A266" s="22" t="s">
         <v>518</v>
       </c>
-      <c r="B266" s="24"/>
+      <c r="B266" s="22"/>
       <c r="C266" s="10">
         <v>4037940.24</v>
       </c>
@@ -16875,10 +16875,10 @@
       </c>
     </row>
     <row r="267" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A267" s="25" t="s">
+      <c r="A267" s="23" t="s">
         <v>519</v>
       </c>
-      <c r="B267" s="25"/>
+      <c r="B267" s="23"/>
       <c r="C267" s="12">
         <v>316919549.19</v>
       </c>
@@ -17321,10 +17321,10 @@
       </c>
     </row>
     <row r="275" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A275" s="22" t="s">
+      <c r="A275" s="24" t="s">
         <v>520</v>
       </c>
-      <c r="B275" s="22"/>
+      <c r="B275" s="24"/>
       <c r="C275" s="15">
         <v>316919549.19</v>
       </c>
@@ -17375,15 +17375,28 @@
       </c>
     </row>
     <row r="276" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="O276" s="23" t="s">
+      <c r="O276" s="25" t="s">
         <v>521</v>
       </c>
-      <c r="P276" s="23"/>
-      <c r="Q276" s="23"/>
-      <c r="R276" s="23"/>
+      <c r="P276" s="25"/>
+      <c r="Q276" s="25"/>
+      <c r="R276" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="Q4:R4"/>
     <mergeCell ref="A266:B266"/>
     <mergeCell ref="A267:B267"/>
     <mergeCell ref="A275:B275"/>
@@ -17393,19 +17406,6 @@
     <mergeCell ref="A257:B257"/>
     <mergeCell ref="A261:B261"/>
     <mergeCell ref="A262:B262"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17437,17 +17437,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+    </row>
+    <row r="4" spans="1:18" ht="31.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>522</v>
       </c>
@@ -19028,10 +19028,10 @@
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A33" s="24" t="s">
+      <c r="A33" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="B33" s="24"/>
+      <c r="B33" s="22"/>
       <c r="C33" s="10">
         <v>220142200</v>
       </c>
@@ -20414,10 +20414,10 @@
       </c>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A58" s="24" t="s">
+      <c r="A58" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="B58" s="24"/>
+      <c r="B58" s="22"/>
       <c r="C58" s="10">
         <v>76013828.769999996</v>
       </c>
@@ -20468,10 +20468,10 @@
       </c>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A59" s="25" t="s">
+      <c r="A59" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="B59" s="25"/>
+      <c r="B59" s="23"/>
       <c r="C59" s="12">
         <v>296156028.76999998</v>
       </c>
@@ -20632,10 +20632,10 @@
       </c>
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A62" s="24" t="s">
+      <c r="A62" s="22" t="s">
         <v>510</v>
       </c>
-      <c r="B62" s="24"/>
+      <c r="B62" s="22"/>
       <c r="C62" s="10">
         <v>16725580.18</v>
       </c>
@@ -20686,10 +20686,10 @@
       </c>
     </row>
     <row r="63" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A63" s="25" t="s">
+      <c r="A63" s="23" t="s">
         <v>511</v>
       </c>
-      <c r="B63" s="25"/>
+      <c r="B63" s="23"/>
       <c r="C63" s="12">
         <v>312881608.94999999</v>
       </c>
@@ -20850,10 +20850,10 @@
       </c>
     </row>
     <row r="66" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A66" s="24" t="s">
+      <c r="A66" s="22" t="s">
         <v>518</v>
       </c>
-      <c r="B66" s="24"/>
+      <c r="B66" s="22"/>
       <c r="C66" s="10">
         <v>4037940.24</v>
       </c>
@@ -20904,10 +20904,10 @@
       </c>
     </row>
     <row r="67" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A67" s="25" t="s">
+      <c r="A67" s="23" t="s">
         <v>519</v>
       </c>
-      <c r="B67" s="25"/>
+      <c r="B67" s="23"/>
       <c r="C67" s="12">
         <v>316919549.19</v>
       </c>
@@ -21498,10 +21498,10 @@
       </c>
     </row>
     <row r="78" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A78" s="22" t="s">
+      <c r="A78" s="24" t="s">
         <v>520</v>
       </c>
-      <c r="B78" s="22"/>
+      <c r="B78" s="24"/>
       <c r="C78" s="15">
         <v>316919549.19</v>
       </c>
@@ -21552,15 +21552,28 @@
       </c>
     </row>
     <row r="79" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="O79" s="23" t="s">
+      <c r="O79" s="25" t="s">
         <v>534</v>
       </c>
-      <c r="P79" s="23"/>
-      <c r="Q79" s="23"/>
-      <c r="R79" s="23"/>
+      <c r="P79" s="25"/>
+      <c r="Q79" s="25"/>
+      <c r="R79" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="O79:R79"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="Q4:R4"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A4:A5"/>
@@ -21570,19 +21583,6 @@
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="A78:B78"/>
-    <mergeCell ref="O79:R79"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A62:B62"/>
-    <mergeCell ref="A63:B63"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A67:B67"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>